<commit_message>
[feat] Projectile 애니메이션 효과 추가 및 Dragon, Enemy SpawnPoint 추가
</commit_message>
<xml_diff>
--- a/ExcelToJsonWizard/excel_files/GameInfo.xlsx
+++ b/ExcelToJsonWizard/excel_files/GameInfo.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="73">
   <si>
     <t>key</t>
   </si>
@@ -22,10 +22,13 @@
     <t>description</t>
   </si>
   <si>
-    <t>spritePath</t>
+    <t>iconPath</t>
   </si>
   <si>
     <t>prefabPath</t>
+  </si>
+  <si>
+    <t>projectileSpritePath</t>
   </si>
   <si>
     <t>drop</t>
@@ -76,6 +79,9 @@
     <t>string</t>
   </si>
   <si>
+    <t>List&lt;string&gt;</t>
+  </si>
+  <si>
     <t>float</t>
   </si>
   <si>
@@ -88,10 +94,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>SpritePath</t>
+    <t>IconPath</t>
   </si>
   <si>
     <t>PrefabPath</t>
+  </si>
+  <si>
+    <t>ProjectileSpritePath</t>
   </si>
   <si>
     <t>Percent</t>
@@ -128,6 +137,9 @@
   </si>
   <si>
     <t>알에서 막 깨어난 용.\n가끔식 자기 똥을 먹는다.</t>
+  </si>
+  <si>
+    <t>Br_baby_00,Br_baby_01</t>
   </si>
   <si>
     <t>어린용</t>
@@ -497,21 +509,22 @@
     <col customWidth="1" min="1" max="1" width="4.0"/>
     <col customWidth="1" min="2" max="2" width="11.88"/>
     <col customWidth="1" min="3" max="3" width="119.25"/>
-    <col customWidth="1" min="4" max="4" width="10.0"/>
+    <col customWidth="1" min="4" max="4" width="8.75"/>
     <col customWidth="1" min="5" max="5" width="10.63"/>
-    <col customWidth="1" min="6" max="6" width="7.38"/>
-    <col customWidth="1" min="7" max="7" width="11.75"/>
-    <col customWidth="1" min="8" max="8" width="10.88"/>
-    <col customWidth="1" min="9" max="9" width="10.5"/>
-    <col customWidth="1" min="10" max="10" width="16.5"/>
-    <col customWidth="1" min="11" max="11" width="17.0"/>
-    <col customWidth="1" min="12" max="12" width="10.63"/>
-    <col customWidth="1" min="13" max="13" width="11.13"/>
-    <col customWidth="1" min="14" max="15" width="10.5"/>
-    <col customWidth="1" min="16" max="16" width="18.0"/>
-    <col customWidth="1" min="17" max="17" width="19.88"/>
-    <col customWidth="1" min="18" max="18" width="17.13"/>
-    <col customWidth="1" min="19" max="19" width="16.25"/>
+    <col customWidth="1" min="6" max="6" width="19.88"/>
+    <col customWidth="1" min="7" max="7" width="7.38"/>
+    <col customWidth="1" min="8" max="8" width="11.75"/>
+    <col customWidth="1" min="9" max="9" width="10.88"/>
+    <col customWidth="1" min="10" max="10" width="10.5"/>
+    <col customWidth="1" min="11" max="11" width="16.5"/>
+    <col customWidth="1" min="12" max="12" width="17.0"/>
+    <col customWidth="1" min="13" max="13" width="10.63"/>
+    <col customWidth="1" min="14" max="14" width="11.13"/>
+    <col customWidth="1" min="15" max="16" width="10.5"/>
+    <col customWidth="1" min="17" max="17" width="18.0"/>
+    <col customWidth="1" min="18" max="18" width="19.88"/>
+    <col customWidth="1" min="19" max="19" width="17.13"/>
+    <col customWidth="1" min="20" max="20" width="16.25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -572,7 +585,9 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2"/>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="U1" s="2"/>
       <c r="V1" s="2"/>
       <c r="W1" s="2"/>
@@ -582,63 +597,65 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="J2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="N2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="O2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="T2" s="5"/>
+        <v>23</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="U2" s="5"/>
       <c r="V2" s="5"/>
       <c r="W2" s="5"/>
@@ -648,63 +665,65 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>29</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="T3" s="5"/>
+        <v>39</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>39</v>
+      </c>
       <c r="U3" s="5"/>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
@@ -717,22 +736,22 @@
         <v>1.0</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1.0</v>
+        <v>41</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="G4" s="3">
         <v>1.0</v>
       </c>
       <c r="H4" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I4" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I4" s="3">
-        <v>1.0</v>
       </c>
       <c r="J4" s="3">
         <v>1.0</v>
@@ -741,13 +760,13 @@
         <v>1.0</v>
       </c>
       <c r="L4" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M4" s="3">
         <v>0.0</v>
       </c>
       <c r="N4" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O4" s="3">
         <v>1.0</v>
@@ -764,7 +783,9 @@
       <c r="S4" s="3">
         <v>1.0</v>
       </c>
-      <c r="T4" s="5"/>
+      <c r="T4" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U4" s="5"/>
       <c r="V4" s="5"/>
       <c r="W4" s="5"/>
@@ -777,22 +798,22 @@
         <v>2.0</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="3">
+        <v>44</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="3">
         <v>1.0</v>
       </c>
-      <c r="G5" s="3">
+      <c r="H5" s="3">
         <v>1.03</v>
       </c>
-      <c r="H5" s="3">
+      <c r="I5" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I5" s="3">
-        <v>1.0</v>
       </c>
       <c r="J5" s="3">
         <v>1.0</v>
@@ -801,13 +822,13 @@
         <v>1.0</v>
       </c>
       <c r="L5" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M5" s="3">
         <v>0.0</v>
       </c>
       <c r="N5" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O5" s="3">
         <v>1.0</v>
@@ -824,7 +845,9 @@
       <c r="S5" s="3">
         <v>1.0</v>
       </c>
-      <c r="T5" s="5"/>
+      <c r="T5" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U5" s="5"/>
       <c r="V5" s="5"/>
       <c r="W5" s="5"/>
@@ -837,22 +860,22 @@
         <v>3.0</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="3">
         <v>1.0</v>
       </c>
-      <c r="G6" s="3">
+      <c r="H6" s="3">
         <v>1.05</v>
       </c>
-      <c r="H6" s="3">
+      <c r="I6" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I6" s="3">
-        <v>1.0</v>
       </c>
       <c r="J6" s="3">
         <v>1.0</v>
@@ -861,13 +884,13 @@
         <v>1.0</v>
       </c>
       <c r="L6" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M6" s="3">
         <v>0.0</v>
       </c>
       <c r="N6" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O6" s="3">
         <v>1.0</v>
@@ -884,7 +907,9 @@
       <c r="S6" s="3">
         <v>1.0</v>
       </c>
-      <c r="T6" s="5"/>
+      <c r="T6" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U6" s="5"/>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
@@ -897,22 +922,22 @@
         <v>4.0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1.0</v>
+        <v>48</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="G7" s="3">
         <v>1.0</v>
       </c>
       <c r="H7" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I7" s="3">
         <v>50.0</v>
-      </c>
-      <c r="I7" s="3">
-        <v>1.0</v>
       </c>
       <c r="J7" s="3">
         <v>1.0</v>
@@ -921,13 +946,13 @@
         <v>1.0</v>
       </c>
       <c r="L7" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M7" s="3">
         <v>0.0</v>
       </c>
       <c r="N7" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O7" s="3">
         <v>1.0</v>
@@ -944,7 +969,9 @@
       <c r="S7" s="3">
         <v>1.0</v>
       </c>
-      <c r="T7" s="5"/>
+      <c r="T7" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U7" s="5"/>
       <c r="V7" s="5"/>
       <c r="W7" s="5"/>
@@ -957,37 +984,37 @@
         <v>5.0</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="3">
-        <v>1.0</v>
+        <v>50</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="G8" s="3">
         <v>1.0</v>
       </c>
       <c r="H8" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I8" s="3">
         <v>0.0</v>
       </c>
-      <c r="I8" s="3">
+      <c r="J8" s="3">
         <v>1.3</v>
-      </c>
-      <c r="J8" s="3">
-        <v>1.0</v>
       </c>
       <c r="K8" s="3">
         <v>1.0</v>
       </c>
       <c r="L8" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M8" s="3">
         <v>0.0</v>
       </c>
       <c r="N8" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O8" s="3">
         <v>1.0</v>
@@ -1004,7 +1031,9 @@
       <c r="S8" s="3">
         <v>1.0</v>
       </c>
-      <c r="T8" s="5"/>
+      <c r="T8" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U8" s="5"/>
       <c r="V8" s="5"/>
       <c r="W8" s="5"/>
@@ -1017,22 +1046,22 @@
         <v>6.0</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F9" s="3">
+        <v>52</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="3">
         <v>0.9</v>
       </c>
-      <c r="G9" s="3">
+      <c r="H9" s="3">
         <v>1.1</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I9" s="3">
-        <v>1.0</v>
       </c>
       <c r="J9" s="3">
         <v>1.0</v>
@@ -1041,13 +1070,13 @@
         <v>1.0</v>
       </c>
       <c r="L9" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M9" s="3">
         <v>0.0</v>
       </c>
       <c r="N9" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O9" s="3">
         <v>1.0</v>
@@ -1064,7 +1093,9 @@
       <c r="S9" s="3">
         <v>1.0</v>
       </c>
-      <c r="T9" s="5"/>
+      <c r="T9" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U9" s="5"/>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
@@ -1077,22 +1108,22 @@
         <v>7.0</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F10" s="3">
+        <v>54</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="3">
         <v>0.9</v>
       </c>
-      <c r="G10" s="3">
+      <c r="H10" s="3">
         <v>1.0</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I10" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I10" s="3">
-        <v>1.0</v>
       </c>
       <c r="J10" s="3">
         <v>1.0</v>
@@ -1101,10 +1132,10 @@
         <v>1.0</v>
       </c>
       <c r="L10" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="M10" s="3">
         <v>0.0</v>
-      </c>
-      <c r="M10" s="3">
-        <v>1.0</v>
       </c>
       <c r="N10" s="3">
         <v>1.0</v>
@@ -1124,7 +1155,9 @@
       <c r="S10" s="3">
         <v>1.0</v>
       </c>
-      <c r="T10" s="5"/>
+      <c r="T10" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U10" s="5"/>
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
@@ -1137,22 +1170,22 @@
         <v>8.0</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F11" s="3">
+        <v>56</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G11" s="3">
         <v>0.9</v>
       </c>
-      <c r="G11" s="3">
+      <c r="H11" s="3">
         <v>1.0</v>
       </c>
-      <c r="H11" s="3">
+      <c r="I11" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I11" s="3">
-        <v>1.0</v>
       </c>
       <c r="J11" s="3">
         <v>1.0</v>
@@ -1161,13 +1194,13 @@
         <v>1.0</v>
       </c>
       <c r="L11" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="M11" s="3">
         <v>-100.0</v>
       </c>
-      <c r="M11" s="3">
+      <c r="N11" s="3">
         <v>0.0</v>
-      </c>
-      <c r="N11" s="3">
-        <v>1.0</v>
       </c>
       <c r="O11" s="3">
         <v>1.0</v>
@@ -1184,7 +1217,9 @@
       <c r="S11" s="3">
         <v>1.0</v>
       </c>
-      <c r="T11" s="5"/>
+      <c r="T11" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U11" s="5"/>
       <c r="V11" s="5"/>
       <c r="W11" s="5"/>
@@ -1197,37 +1232,37 @@
         <v>9.0</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" s="3">
+        <v>58</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G12" s="3">
         <v>0.9</v>
       </c>
-      <c r="G12" s="3">
+      <c r="H12" s="3">
         <v>1.0</v>
       </c>
-      <c r="H12" s="3">
+      <c r="I12" s="3">
         <v>0.0</v>
       </c>
-      <c r="I12" s="3">
+      <c r="J12" s="3">
         <v>1.0</v>
       </c>
-      <c r="J12" s="3">
+      <c r="K12" s="3">
         <v>1.5</v>
       </c>
-      <c r="K12" s="3">
+      <c r="L12" s="3">
         <v>2.0</v>
-      </c>
-      <c r="L12" s="3">
-        <v>0.0</v>
       </c>
       <c r="M12" s="3">
         <v>0.0</v>
       </c>
       <c r="N12" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O12" s="3">
         <v>1.0</v>
@@ -1244,7 +1279,9 @@
       <c r="S12" s="3">
         <v>1.0</v>
       </c>
-      <c r="T12" s="5"/>
+      <c r="T12" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U12" s="5"/>
       <c r="V12" s="5"/>
       <c r="W12" s="5"/>
@@ -1257,37 +1294,37 @@
         <v>10.0</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" s="3">
+        <v>60</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" s="3">
         <v>0.8</v>
       </c>
-      <c r="G13" s="3">
+      <c r="H13" s="3">
         <v>1.0</v>
       </c>
-      <c r="H13" s="3">
+      <c r="I13" s="3">
         <v>0.0</v>
       </c>
-      <c r="I13" s="3">
+      <c r="J13" s="3">
         <v>1.0</v>
       </c>
-      <c r="J13" s="3">
+      <c r="K13" s="3">
         <v>1.8</v>
       </c>
-      <c r="K13" s="3">
+      <c r="L13" s="3">
         <v>2.3</v>
-      </c>
-      <c r="L13" s="3">
-        <v>0.0</v>
       </c>
       <c r="M13" s="3">
         <v>0.0</v>
       </c>
       <c r="N13" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O13" s="3">
         <v>1.0</v>
@@ -1304,7 +1341,9 @@
       <c r="S13" s="3">
         <v>1.0</v>
       </c>
-      <c r="T13" s="5"/>
+      <c r="T13" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U13" s="5"/>
       <c r="V13" s="5"/>
       <c r="W13" s="5"/>
@@ -1317,22 +1356,22 @@
         <v>11.0</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F14" s="3">
+        <v>62</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" s="3">
         <v>0.8</v>
       </c>
-      <c r="G14" s="3">
+      <c r="H14" s="3">
         <v>1.0</v>
       </c>
-      <c r="H14" s="3">
+      <c r="I14" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I14" s="3">
-        <v>1.0</v>
       </c>
       <c r="J14" s="3">
         <v>1.0</v>
@@ -1341,16 +1380,16 @@
         <v>1.0</v>
       </c>
       <c r="L14" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M14" s="3">
         <v>0.0</v>
       </c>
       <c r="N14" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="O14" s="3">
         <v>1.1</v>
-      </c>
-      <c r="O14" s="3">
-        <v>1.0</v>
       </c>
       <c r="P14" s="3">
         <v>1.0</v>
@@ -1364,7 +1403,9 @@
       <c r="S14" s="3">
         <v>1.0</v>
       </c>
-      <c r="T14" s="5"/>
+      <c r="T14" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U14" s="5"/>
       <c r="V14" s="5"/>
       <c r="W14" s="5"/>
@@ -1377,37 +1418,37 @@
         <v>12.0</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F15" s="3">
+        <v>64</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G15" s="3">
         <v>0.8</v>
       </c>
-      <c r="G15" s="3">
+      <c r="H15" s="3">
         <v>1.0</v>
       </c>
-      <c r="H15" s="3">
+      <c r="I15" s="3">
         <v>0.0</v>
       </c>
-      <c r="I15" s="3">
+      <c r="J15" s="3">
         <v>1.4</v>
-      </c>
-      <c r="J15" s="3">
-        <v>1.0</v>
       </c>
       <c r="K15" s="3">
         <v>1.0</v>
       </c>
       <c r="L15" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M15" s="3">
         <v>0.0</v>
       </c>
       <c r="N15" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O15" s="3">
         <v>1.0</v>
@@ -1424,7 +1465,9 @@
       <c r="S15" s="3">
         <v>1.0</v>
       </c>
-      <c r="T15" s="5"/>
+      <c r="T15" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U15" s="5"/>
       <c r="V15" s="5"/>
       <c r="W15" s="5"/>
@@ -1437,22 +1480,22 @@
         <v>13.0</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="F16" s="3">
+        <v>66</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G16" s="3">
         <v>0.8</v>
       </c>
-      <c r="G16" s="3">
+      <c r="H16" s="3">
         <v>1.0</v>
       </c>
-      <c r="H16" s="3">
+      <c r="I16" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I16" s="3">
-        <v>1.0</v>
       </c>
       <c r="J16" s="3">
         <v>1.0</v>
@@ -1461,19 +1504,19 @@
         <v>1.0</v>
       </c>
       <c r="L16" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M16" s="3">
         <v>0.0</v>
       </c>
       <c r="N16" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="O16" s="3">
         <v>1.0</v>
       </c>
-      <c r="O16" s="3">
+      <c r="P16" s="3">
         <v>1.5</v>
-      </c>
-      <c r="P16" s="3">
-        <v>1.0</v>
       </c>
       <c r="Q16" s="3">
         <v>1.0</v>
@@ -1484,7 +1527,9 @@
       <c r="S16" s="3">
         <v>1.0</v>
       </c>
-      <c r="T16" s="5"/>
+      <c r="T16" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U16" s="5"/>
       <c r="V16" s="5"/>
       <c r="W16" s="5"/>
@@ -1497,22 +1542,22 @@
         <v>14.0</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="F17" s="3">
+        <v>68</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" s="3">
         <v>0.8</v>
       </c>
-      <c r="G17" s="3">
+      <c r="H17" s="3">
         <v>1.0</v>
       </c>
-      <c r="H17" s="3">
+      <c r="I17" s="3">
         <v>100.0</v>
-      </c>
-      <c r="I17" s="3">
-        <v>1.0</v>
       </c>
       <c r="J17" s="3">
         <v>1.0</v>
@@ -1521,13 +1566,13 @@
         <v>1.0</v>
       </c>
       <c r="L17" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M17" s="3">
         <v>0.0</v>
       </c>
       <c r="N17" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O17" s="3">
         <v>1.0</v>
@@ -1544,7 +1589,9 @@
       <c r="S17" s="3">
         <v>1.0</v>
       </c>
-      <c r="T17" s="5"/>
+      <c r="T17" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U17" s="5"/>
       <c r="V17" s="5"/>
       <c r="W17" s="5"/>
@@ -1557,22 +1604,22 @@
         <v>15.0</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="3">
+        <v>70</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G18" s="3">
         <v>0.8</v>
       </c>
-      <c r="G18" s="3">
+      <c r="H18" s="3">
         <v>1.15</v>
       </c>
-      <c r="H18" s="3">
+      <c r="I18" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I18" s="3">
-        <v>1.0</v>
       </c>
       <c r="J18" s="3">
         <v>1.0</v>
@@ -1581,13 +1628,13 @@
         <v>1.0</v>
       </c>
       <c r="L18" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M18" s="3">
         <v>0.0</v>
       </c>
       <c r="N18" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O18" s="3">
         <v>1.0</v>
@@ -1604,7 +1651,9 @@
       <c r="S18" s="3">
         <v>1.0</v>
       </c>
-      <c r="T18" s="5"/>
+      <c r="T18" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U18" s="5"/>
       <c r="V18" s="5"/>
       <c r="W18" s="5"/>
@@ -1617,22 +1666,22 @@
         <v>16.0</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F19" s="3">
+        <v>72</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G19" s="3">
         <v>0.8</v>
       </c>
-      <c r="G19" s="3">
+      <c r="H19" s="3">
         <v>1.3</v>
       </c>
-      <c r="H19" s="3">
+      <c r="I19" s="3">
         <v>0.0</v>
-      </c>
-      <c r="I19" s="3">
-        <v>1.0</v>
       </c>
       <c r="J19" s="3">
         <v>1.0</v>
@@ -1641,13 +1690,13 @@
         <v>1.0</v>
       </c>
       <c r="L19" s="3">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="M19" s="3">
         <v>0.0</v>
       </c>
       <c r="N19" s="3">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O19" s="3">
         <v>1.0</v>
@@ -1664,7 +1713,9 @@
       <c r="S19" s="3">
         <v>1.0</v>
       </c>
-      <c r="T19" s="5"/>
+      <c r="T19" s="3">
+        <v>1.0</v>
+      </c>
       <c r="U19" s="5"/>
       <c r="V19" s="5"/>
       <c r="W19" s="5"/>

</xml_diff>